<commit_message>
Removed unused live monitoring template sheet
</commit_message>
<xml_diff>
--- a/tender_input_master_final.xlsx
+++ b/tender_input_master_final.xlsx
@@ -4,22 +4,21 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="204" yWindow="588" windowWidth="22716" windowHeight="8676"/>
+    <workbookView xWindow="204" yWindow="588" windowWidth="22716" windowHeight="8676" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="officers" sheetId="1" r:id="rId1"/>
     <sheet name="approvers" sheetId="2" r:id="rId2"/>
     <sheet name="config" sheetId="3" r:id="rId3"/>
     <sheet name="tender_master" sheetId="4" r:id="rId4"/>
-    <sheet name="live_monitoring_template" sheetId="5" r:id="rId5"/>
-    <sheet name="summary_check" sheetId="6" r:id="rId6"/>
+    <sheet name="summary_check" sheetId="6" r:id="rId5"/>
   </sheets>
   <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3072" uniqueCount="518">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3061" uniqueCount="512">
   <si>
     <t>officer_id</t>
   </si>
@@ -1483,24 +1482,6 @@
   </si>
   <si>
     <t>2026-07-06</t>
-  </si>
-  <si>
-    <t>Current Stage</t>
-  </si>
-  <si>
-    <t>Pending With</t>
-  </si>
-  <si>
-    <t>Planned Date</t>
-  </si>
-  <si>
-    <t>Actual Date</t>
-  </si>
-  <si>
-    <t>Delay Days</t>
-  </si>
-  <si>
-    <t>SLA Status</t>
   </si>
   <si>
     <t>Check</t>
@@ -1860,7 +1841,7 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>505</v>
+        <v>499</v>
       </c>
       <c r="B2" t="s">
         <v>5</v>
@@ -1877,7 +1858,7 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>506</v>
+        <v>500</v>
       </c>
       <c r="B3" t="s">
         <v>9</v>
@@ -1894,7 +1875,7 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>507</v>
+        <v>501</v>
       </c>
       <c r="B4" t="s">
         <v>11</v>
@@ -1911,7 +1892,7 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>508</v>
+        <v>502</v>
       </c>
       <c r="B5" t="s">
         <v>14</v>
@@ -1928,7 +1909,7 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>509</v>
+        <v>503</v>
       </c>
       <c r="B6" t="s">
         <v>16</v>
@@ -1945,7 +1926,7 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>510</v>
+        <v>504</v>
       </c>
       <c r="B7" t="s">
         <v>17</v>
@@ -1962,7 +1943,7 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>511</v>
+        <v>505</v>
       </c>
       <c r="B8" t="s">
         <v>18</v>
@@ -1979,7 +1960,7 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>512</v>
+        <v>506</v>
       </c>
       <c r="B9" t="s">
         <v>19</v>
@@ -1996,7 +1977,7 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>513</v>
+        <v>507</v>
       </c>
       <c r="B10" t="s">
         <v>20</v>
@@ -2013,7 +1994,7 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>514</v>
+        <v>508</v>
       </c>
       <c r="B11" t="s">
         <v>21</v>
@@ -2064,7 +2045,7 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>515</v>
+        <v>509</v>
       </c>
       <c r="B2" t="s">
         <v>27</v>
@@ -2081,7 +2062,7 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>516</v>
+        <v>510</v>
       </c>
       <c r="B3" t="s">
         <v>30</v>
@@ -2098,7 +2079,7 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>517</v>
+        <v>511</v>
       </c>
       <c r="B4" t="s">
         <v>33</v>
@@ -2366,7 +2347,7 @@
         <v>81</v>
       </c>
       <c r="C2" t="s">
-        <v>511</v>
+        <v>505</v>
       </c>
       <c r="D2">
         <v>2098.14</v>
@@ -2446,7 +2427,7 @@
         <v>22</v>
       </c>
       <c r="C3" t="s">
-        <v>509</v>
+        <v>503</v>
       </c>
       <c r="D3">
         <v>14.05</v>
@@ -2485,7 +2466,7 @@
         <v>8</v>
       </c>
       <c r="C4" t="s">
-        <v>505</v>
+        <v>499</v>
       </c>
       <c r="D4">
         <v>14.26</v>
@@ -2560,7 +2541,7 @@
         <v>8</v>
       </c>
       <c r="C5" t="s">
-        <v>505</v>
+        <v>499</v>
       </c>
       <c r="D5">
         <v>86.97</v>
@@ -2633,7 +2614,7 @@
         <v>8</v>
       </c>
       <c r="C6" t="s">
-        <v>507</v>
+        <v>501</v>
       </c>
       <c r="D6">
         <v>625.35</v>
@@ -2708,7 +2689,7 @@
         <v>8</v>
       </c>
       <c r="C7" t="s">
-        <v>507</v>
+        <v>501</v>
       </c>
       <c r="D7">
         <v>697.47</v>
@@ -2783,7 +2764,7 @@
         <v>8</v>
       </c>
       <c r="C8" t="s">
-        <v>506</v>
+        <v>500</v>
       </c>
       <c r="D8">
         <v>14.71</v>
@@ -2858,7 +2839,7 @@
         <v>8</v>
       </c>
       <c r="C9" t="s">
-        <v>506</v>
+        <v>500</v>
       </c>
       <c r="D9">
         <v>943.99</v>
@@ -2931,7 +2912,7 @@
         <v>22</v>
       </c>
       <c r="C10" t="s">
-        <v>513</v>
+        <v>507</v>
       </c>
       <c r="D10">
         <v>716.91</v>
@@ -3006,7 +2987,7 @@
         <v>22</v>
       </c>
       <c r="C11" t="s">
-        <v>512</v>
+        <v>506</v>
       </c>
       <c r="D11">
         <v>863.78</v>
@@ -3081,7 +3062,7 @@
         <v>22</v>
       </c>
       <c r="C12" t="s">
-        <v>508</v>
+        <v>502</v>
       </c>
       <c r="D12">
         <v>706.02</v>
@@ -3156,7 +3137,7 @@
         <v>22</v>
       </c>
       <c r="C13" t="s">
-        <v>514</v>
+        <v>508</v>
       </c>
       <c r="D13">
         <v>706.72</v>
@@ -3215,7 +3196,7 @@
         <v>8</v>
       </c>
       <c r="C14" t="s">
-        <v>506</v>
+        <v>500</v>
       </c>
       <c r="D14">
         <v>549.6</v>
@@ -3295,7 +3276,7 @@
         <v>81</v>
       </c>
       <c r="C15" t="s">
-        <v>509</v>
+        <v>503</v>
       </c>
       <c r="D15">
         <v>431.37</v>
@@ -3375,7 +3356,7 @@
         <v>22</v>
       </c>
       <c r="C16" t="s">
-        <v>512</v>
+        <v>506</v>
       </c>
       <c r="D16">
         <v>3990.98</v>
@@ -3455,7 +3436,7 @@
         <v>8</v>
       </c>
       <c r="C17" t="s">
-        <v>506</v>
+        <v>500</v>
       </c>
       <c r="D17">
         <v>77.86</v>
@@ -3530,7 +3511,7 @@
         <v>8</v>
       </c>
       <c r="C18" t="s">
-        <v>506</v>
+        <v>500</v>
       </c>
       <c r="D18">
         <v>1713.92</v>
@@ -3610,7 +3591,7 @@
         <v>22</v>
       </c>
       <c r="C19" t="s">
-        <v>514</v>
+        <v>508</v>
       </c>
       <c r="D19">
         <v>36.15</v>
@@ -3685,7 +3666,7 @@
         <v>22</v>
       </c>
       <c r="C20" t="s">
-        <v>509</v>
+        <v>503</v>
       </c>
       <c r="D20">
         <v>655.16</v>
@@ -3731,7 +3712,7 @@
         <v>22</v>
       </c>
       <c r="C21" t="s">
-        <v>513</v>
+        <v>507</v>
       </c>
       <c r="D21">
         <v>7911.02</v>
@@ -3811,7 +3792,7 @@
         <v>22</v>
       </c>
       <c r="C22" t="s">
-        <v>508</v>
+        <v>502</v>
       </c>
       <c r="D22">
         <v>98.29</v>
@@ -3886,7 +3867,7 @@
         <v>8</v>
       </c>
       <c r="C23" t="s">
-        <v>505</v>
+        <v>499</v>
       </c>
       <c r="D23">
         <v>640.91</v>
@@ -3961,7 +3942,7 @@
         <v>22</v>
       </c>
       <c r="C24" t="s">
-        <v>512</v>
+        <v>506</v>
       </c>
       <c r="D24">
         <v>664.33</v>
@@ -4034,7 +4015,7 @@
         <v>8</v>
       </c>
       <c r="C25" t="s">
-        <v>506</v>
+        <v>500</v>
       </c>
       <c r="D25">
         <v>181.47</v>
@@ -4109,7 +4090,7 @@
         <v>81</v>
       </c>
       <c r="C26" t="s">
-        <v>509</v>
+        <v>503</v>
       </c>
       <c r="D26">
         <v>531.84</v>
@@ -4189,7 +4170,7 @@
         <v>22</v>
       </c>
       <c r="C27" t="s">
-        <v>512</v>
+        <v>506</v>
       </c>
       <c r="D27">
         <v>26.15</v>
@@ -4269,7 +4250,7 @@
         <v>8</v>
       </c>
       <c r="C28" t="s">
-        <v>505</v>
+        <v>499</v>
       </c>
       <c r="D28">
         <v>92.89</v>
@@ -4338,7 +4319,7 @@
         <v>22</v>
       </c>
       <c r="C29" t="s">
-        <v>514</v>
+        <v>508</v>
       </c>
       <c r="D29">
         <v>33.35</v>
@@ -4418,7 +4399,7 @@
         <v>8</v>
       </c>
       <c r="C30" t="s">
-        <v>506</v>
+        <v>500</v>
       </c>
       <c r="D30">
         <v>976.29</v>
@@ -4480,7 +4461,7 @@
         <v>8</v>
       </c>
       <c r="C31" t="s">
-        <v>507</v>
+        <v>501</v>
       </c>
       <c r="D31">
         <v>167.55</v>
@@ -4553,7 +4534,7 @@
         <v>8</v>
       </c>
       <c r="C32" t="s">
-        <v>506</v>
+        <v>500</v>
       </c>
       <c r="D32">
         <v>87.24</v>
@@ -4626,7 +4607,7 @@
         <v>22</v>
       </c>
       <c r="C33" t="s">
-        <v>510</v>
+        <v>504</v>
       </c>
       <c r="D33">
         <v>665</v>
@@ -4675,7 +4656,7 @@
         <v>22</v>
       </c>
       <c r="C34" t="s">
-        <v>509</v>
+        <v>503</v>
       </c>
       <c r="D34">
         <v>65.989999999999995</v>
@@ -4721,7 +4702,7 @@
         <v>81</v>
       </c>
       <c r="C35" t="s">
-        <v>508</v>
+        <v>502</v>
       </c>
       <c r="D35">
         <v>523.4</v>
@@ -4801,7 +4782,7 @@
         <v>8</v>
       </c>
       <c r="C36" t="s">
-        <v>507</v>
+        <v>501</v>
       </c>
       <c r="D36">
         <v>863.14</v>
@@ -4876,7 +4857,7 @@
         <v>22</v>
       </c>
       <c r="C37" t="s">
-        <v>511</v>
+        <v>505</v>
       </c>
       <c r="D37">
         <v>432.19</v>
@@ -4949,7 +4930,7 @@
         <v>81</v>
       </c>
       <c r="C38" t="s">
-        <v>511</v>
+        <v>505</v>
       </c>
       <c r="D38">
         <v>68.55</v>
@@ -5024,7 +5005,7 @@
         <v>22</v>
       </c>
       <c r="C39" t="s">
-        <v>509</v>
+        <v>503</v>
       </c>
       <c r="D39">
         <v>54.85</v>
@@ -5104,7 +5085,7 @@
         <v>22</v>
       </c>
       <c r="C40" t="s">
-        <v>511</v>
+        <v>505</v>
       </c>
       <c r="D40">
         <v>512.28</v>
@@ -5177,7 +5158,7 @@
         <v>81</v>
       </c>
       <c r="C41" t="s">
-        <v>508</v>
+        <v>502</v>
       </c>
       <c r="D41">
         <v>16.3</v>
@@ -5223,7 +5204,7 @@
         <v>22</v>
       </c>
       <c r="C42" t="s">
-        <v>511</v>
+        <v>505</v>
       </c>
       <c r="D42">
         <v>7676.96</v>
@@ -5296,7 +5277,7 @@
         <v>22</v>
       </c>
       <c r="C43" t="s">
-        <v>510</v>
+        <v>504</v>
       </c>
       <c r="D43">
         <v>88.36</v>
@@ -5371,7 +5352,7 @@
         <v>22</v>
       </c>
       <c r="C44" t="s">
-        <v>508</v>
+        <v>502</v>
       </c>
       <c r="D44">
         <v>568.09</v>
@@ -5451,7 +5432,7 @@
         <v>8</v>
       </c>
       <c r="C45" t="s">
-        <v>507</v>
+        <v>501</v>
       </c>
       <c r="D45">
         <v>85.51</v>
@@ -5527,7 +5508,7 @@
         <v>81</v>
       </c>
       <c r="C46" t="s">
-        <v>509</v>
+        <v>503</v>
       </c>
       <c r="D46">
         <v>18.100000000000001</v>
@@ -5602,7 +5583,7 @@
         <v>8</v>
       </c>
       <c r="C47" t="s">
-        <v>505</v>
+        <v>499</v>
       </c>
       <c r="D47">
         <v>678.51</v>
@@ -5653,7 +5634,7 @@
         <v>8</v>
       </c>
       <c r="C48" t="s">
-        <v>507</v>
+        <v>501</v>
       </c>
       <c r="D48">
         <v>88.77</v>
@@ -5726,7 +5707,7 @@
         <v>22</v>
       </c>
       <c r="C49" t="s">
-        <v>513</v>
+        <v>507</v>
       </c>
       <c r="D49">
         <v>53.24</v>
@@ -5787,7 +5768,7 @@
         <v>22</v>
       </c>
       <c r="C50" t="s">
-        <v>508</v>
+        <v>502</v>
       </c>
       <c r="D50">
         <v>854.73</v>
@@ -5862,7 +5843,7 @@
         <v>22</v>
       </c>
       <c r="C51" t="s">
-        <v>513</v>
+        <v>507</v>
       </c>
       <c r="D51">
         <v>293.79000000000002</v>
@@ -5937,7 +5918,7 @@
         <v>22</v>
       </c>
       <c r="C52" t="s">
-        <v>512</v>
+        <v>506</v>
       </c>
       <c r="D52">
         <v>655.5</v>
@@ -6010,7 +5991,7 @@
         <v>8</v>
       </c>
       <c r="C53" t="s">
-        <v>505</v>
+        <v>499</v>
       </c>
       <c r="D53">
         <v>7002.32</v>
@@ -6085,7 +6066,7 @@
         <v>22</v>
       </c>
       <c r="C54" t="s">
-        <v>512</v>
+        <v>506</v>
       </c>
       <c r="D54">
         <v>538.08000000000004</v>
@@ -6158,7 +6139,7 @@
         <v>22</v>
       </c>
       <c r="C55" t="s">
-        <v>511</v>
+        <v>505</v>
       </c>
       <c r="D55">
         <v>64.89</v>
@@ -6202,7 +6183,7 @@
         <v>22</v>
       </c>
       <c r="C56" t="s">
-        <v>508</v>
+        <v>502</v>
       </c>
       <c r="D56">
         <v>905.81</v>
@@ -6277,7 +6258,7 @@
         <v>22</v>
       </c>
       <c r="C57" t="s">
-        <v>514</v>
+        <v>508</v>
       </c>
       <c r="D57">
         <v>7354.6</v>
@@ -6352,7 +6333,7 @@
         <v>22</v>
       </c>
       <c r="C58" t="s">
-        <v>508</v>
+        <v>502</v>
       </c>
       <c r="D58">
         <v>778.96</v>
@@ -6427,7 +6408,7 @@
         <v>81</v>
       </c>
       <c r="C59" t="s">
-        <v>513</v>
+        <v>507</v>
       </c>
       <c r="D59">
         <v>9623.26</v>
@@ -6507,7 +6488,7 @@
         <v>22</v>
       </c>
       <c r="C60" t="s">
-        <v>513</v>
+        <v>507</v>
       </c>
       <c r="D60">
         <v>775.93</v>
@@ -6548,7 +6529,7 @@
         <v>22</v>
       </c>
       <c r="C61" t="s">
-        <v>511</v>
+        <v>505</v>
       </c>
       <c r="D61">
         <v>52.92</v>
@@ -6617,7 +6598,7 @@
         <v>8</v>
       </c>
       <c r="C62" t="s">
-        <v>506</v>
+        <v>500</v>
       </c>
       <c r="D62">
         <v>15.77</v>
@@ -6654,7 +6635,7 @@
         <v>22</v>
       </c>
       <c r="C63" t="s">
-        <v>509</v>
+        <v>503</v>
       </c>
       <c r="D63">
         <v>176.73</v>
@@ -6729,7 +6710,7 @@
         <v>22</v>
       </c>
       <c r="C64" t="s">
-        <v>512</v>
+        <v>506</v>
       </c>
       <c r="D64">
         <v>941.03</v>
@@ -6804,7 +6785,7 @@
         <v>22</v>
       </c>
       <c r="C65" t="s">
-        <v>508</v>
+        <v>502</v>
       </c>
       <c r="D65">
         <v>594.95000000000005</v>
@@ -6879,7 +6860,7 @@
         <v>8</v>
       </c>
       <c r="C66" t="s">
-        <v>506</v>
+        <v>500</v>
       </c>
       <c r="D66">
         <v>652.33000000000004</v>
@@ -6959,7 +6940,7 @@
         <v>22</v>
       </c>
       <c r="C67" t="s">
-        <v>514</v>
+        <v>508</v>
       </c>
       <c r="D67">
         <v>96.34</v>
@@ -7034,7 +7015,7 @@
         <v>22</v>
       </c>
       <c r="C68" t="s">
-        <v>512</v>
+        <v>506</v>
       </c>
       <c r="D68">
         <v>3150</v>
@@ -7109,7 +7090,7 @@
         <v>22</v>
       </c>
       <c r="C69" t="s">
-        <v>512</v>
+        <v>506</v>
       </c>
       <c r="D69">
         <v>225.65</v>
@@ -7184,7 +7165,7 @@
         <v>22</v>
       </c>
       <c r="C70" t="s">
-        <v>512</v>
+        <v>506</v>
       </c>
       <c r="D70">
         <v>15.89</v>
@@ -7264,7 +7245,7 @@
         <v>22</v>
       </c>
       <c r="C71" t="s">
-        <v>511</v>
+        <v>505</v>
       </c>
       <c r="D71">
         <v>53.72</v>
@@ -7339,7 +7320,7 @@
         <v>22</v>
       </c>
       <c r="C72" t="s">
-        <v>509</v>
+        <v>503</v>
       </c>
       <c r="D72">
         <v>434.99</v>
@@ -7414,7 +7395,7 @@
         <v>22</v>
       </c>
       <c r="C73" t="s">
-        <v>509</v>
+        <v>503</v>
       </c>
       <c r="D73">
         <v>172.59</v>
@@ -7494,7 +7475,7 @@
         <v>22</v>
       </c>
       <c r="C74" t="s">
-        <v>512</v>
+        <v>506</v>
       </c>
       <c r="D74">
         <v>56.49</v>
@@ -7569,7 +7550,7 @@
         <v>8</v>
       </c>
       <c r="C75" t="s">
-        <v>505</v>
+        <v>499</v>
       </c>
       <c r="D75">
         <v>5830.49</v>
@@ -7642,7 +7623,7 @@
         <v>22</v>
       </c>
       <c r="C76" t="s">
-        <v>510</v>
+        <v>504</v>
       </c>
       <c r="D76">
         <v>684.38</v>
@@ -7717,7 +7698,7 @@
         <v>22</v>
       </c>
       <c r="C77" t="s">
-        <v>508</v>
+        <v>502</v>
       </c>
       <c r="D77">
         <v>80.31</v>
@@ -7792,7 +7773,7 @@
         <v>22</v>
       </c>
       <c r="C78" t="s">
-        <v>508</v>
+        <v>502</v>
       </c>
       <c r="D78">
         <v>666.13</v>
@@ -7865,7 +7846,7 @@
         <v>22</v>
       </c>
       <c r="C79" t="s">
-        <v>514</v>
+        <v>508</v>
       </c>
       <c r="D79">
         <v>92.95</v>
@@ -7938,7 +7919,7 @@
         <v>22</v>
       </c>
       <c r="C80" t="s">
-        <v>514</v>
+        <v>508</v>
       </c>
       <c r="D80">
         <v>858.76</v>
@@ -8011,7 +7992,7 @@
         <v>22</v>
       </c>
       <c r="C81" t="s">
-        <v>514</v>
+        <v>508</v>
       </c>
       <c r="D81">
         <v>578.70000000000005</v>
@@ -8086,7 +8067,7 @@
         <v>8</v>
       </c>
       <c r="C82" t="s">
-        <v>507</v>
+        <v>501</v>
       </c>
       <c r="D82">
         <v>670.67</v>
@@ -8161,7 +8142,7 @@
         <v>8</v>
       </c>
       <c r="C83" t="s">
-        <v>507</v>
+        <v>501</v>
       </c>
       <c r="D83">
         <v>6927.75</v>
@@ -8236,7 +8217,7 @@
         <v>22</v>
       </c>
       <c r="C84" t="s">
-        <v>514</v>
+        <v>508</v>
       </c>
       <c r="D84">
         <v>2427</v>
@@ -8311,7 +8292,7 @@
         <v>22</v>
       </c>
       <c r="C85" t="s">
-        <v>510</v>
+        <v>504</v>
       </c>
       <c r="D85">
         <v>3453.12</v>
@@ -8391,7 +8372,7 @@
         <v>22</v>
       </c>
       <c r="C86" t="s">
-        <v>513</v>
+        <v>507</v>
       </c>
       <c r="D86">
         <v>3953.43</v>
@@ -8466,7 +8447,7 @@
         <v>22</v>
       </c>
       <c r="C87" t="s">
-        <v>513</v>
+        <v>507</v>
       </c>
       <c r="D87">
         <v>72.89</v>
@@ -8541,7 +8522,7 @@
         <v>22</v>
       </c>
       <c r="C88" t="s">
-        <v>510</v>
+        <v>504</v>
       </c>
       <c r="D88">
         <v>537.45000000000005</v>
@@ -8616,7 +8597,7 @@
         <v>8</v>
       </c>
       <c r="C89" t="s">
-        <v>507</v>
+        <v>501</v>
       </c>
       <c r="D89">
         <v>902.64</v>
@@ -8689,7 +8670,7 @@
         <v>22</v>
       </c>
       <c r="C90" t="s">
-        <v>513</v>
+        <v>507</v>
       </c>
       <c r="D90">
         <v>2316.87</v>
@@ -8764,7 +8745,7 @@
         <v>22</v>
       </c>
       <c r="C91" t="s">
-        <v>510</v>
+        <v>504</v>
       </c>
       <c r="D91">
         <v>10.48</v>
@@ -8803,7 +8784,7 @@
         <v>22</v>
       </c>
       <c r="C92" t="s">
-        <v>513</v>
+        <v>507</v>
       </c>
       <c r="D92">
         <v>364.15</v>
@@ -8865,7 +8846,7 @@
         <v>8</v>
       </c>
       <c r="C93" t="s">
-        <v>507</v>
+        <v>501</v>
       </c>
       <c r="D93">
         <v>70.22</v>
@@ -8924,7 +8905,7 @@
         <v>8</v>
       </c>
       <c r="C94" t="s">
-        <v>507</v>
+        <v>501</v>
       </c>
       <c r="D94">
         <v>355.87</v>
@@ -8999,7 +8980,7 @@
         <v>8</v>
       </c>
       <c r="C95" t="s">
-        <v>507</v>
+        <v>501</v>
       </c>
       <c r="D95">
         <v>78.59</v>
@@ -9074,7 +9055,7 @@
         <v>22</v>
       </c>
       <c r="C96" t="s">
-        <v>513</v>
+        <v>507</v>
       </c>
       <c r="D96">
         <v>304.95999999999998</v>
@@ -9148,7 +9129,7 @@
         <v>8</v>
       </c>
       <c r="C97" t="s">
-        <v>506</v>
+        <v>500</v>
       </c>
       <c r="D97">
         <v>78.37</v>
@@ -9217,7 +9198,7 @@
         <v>22</v>
       </c>
       <c r="C98" t="s">
-        <v>513</v>
+        <v>507</v>
       </c>
       <c r="D98">
         <v>418.51</v>
@@ -9293,7 +9274,7 @@
         <v>81</v>
       </c>
       <c r="C99" t="s">
-        <v>508</v>
+        <v>502</v>
       </c>
       <c r="D99">
         <v>32.119999999999997</v>
@@ -9364,7 +9345,7 @@
         <v>22</v>
       </c>
       <c r="C100" t="s">
-        <v>508</v>
+        <v>502</v>
       </c>
       <c r="D100">
         <v>703.23</v>
@@ -9437,7 +9418,7 @@
         <v>22</v>
       </c>
       <c r="C101" t="s">
-        <v>510</v>
+        <v>504</v>
       </c>
       <c r="D101">
         <v>11.25</v>
@@ -9506,7 +9487,7 @@
         <v>22</v>
       </c>
       <c r="C102" t="s">
-        <v>510</v>
+        <v>504</v>
       </c>
       <c r="D102">
         <v>434.26</v>
@@ -9575,7 +9556,7 @@
         <v>22</v>
       </c>
       <c r="C103" t="s">
-        <v>510</v>
+        <v>504</v>
       </c>
       <c r="D103">
         <v>402.46</v>
@@ -9644,7 +9625,7 @@
         <v>22</v>
       </c>
       <c r="C104" t="s">
-        <v>514</v>
+        <v>508</v>
       </c>
       <c r="D104">
         <v>695.56</v>
@@ -9705,7 +9686,7 @@
         <v>81</v>
       </c>
       <c r="C105" t="s">
-        <v>508</v>
+        <v>502</v>
       </c>
       <c r="D105">
         <v>9463.5400000000009</v>
@@ -9779,7 +9760,7 @@
         <v>22</v>
       </c>
       <c r="C106" t="s">
-        <v>513</v>
+        <v>507</v>
       </c>
       <c r="D106">
         <v>65.88</v>
@@ -9848,7 +9829,7 @@
         <v>22</v>
       </c>
       <c r="C107" t="s">
-        <v>508</v>
+        <v>502</v>
       </c>
       <c r="D107">
         <v>589.29</v>
@@ -9897,7 +9878,7 @@
         <v>8</v>
       </c>
       <c r="C108" t="s">
-        <v>505</v>
+        <v>499</v>
       </c>
       <c r="D108">
         <v>53.38</v>
@@ -9972,7 +9953,7 @@
         <v>22</v>
       </c>
       <c r="C109" t="s">
-        <v>510</v>
+        <v>504</v>
       </c>
       <c r="D109">
         <v>40.28</v>
@@ -10041,7 +10022,7 @@
         <v>22</v>
       </c>
       <c r="C110" t="s">
-        <v>509</v>
+        <v>503</v>
       </c>
       <c r="D110">
         <v>22.91</v>
@@ -10116,7 +10097,7 @@
         <v>22</v>
       </c>
       <c r="C111" t="s">
-        <v>508</v>
+        <v>502</v>
       </c>
       <c r="D111">
         <v>525.97</v>
@@ -10177,7 +10158,7 @@
         <v>22</v>
       </c>
       <c r="C112" t="s">
-        <v>514</v>
+        <v>508</v>
       </c>
       <c r="D112">
         <v>18.61</v>
@@ -10257,7 +10238,7 @@
         <v>8</v>
       </c>
       <c r="C113" t="s">
-        <v>507</v>
+        <v>501</v>
       </c>
       <c r="D113">
         <v>98.9</v>
@@ -10332,7 +10313,7 @@
         <v>8</v>
       </c>
       <c r="C114" t="s">
-        <v>506</v>
+        <v>500</v>
       </c>
       <c r="D114">
         <v>553.5</v>
@@ -10405,7 +10386,7 @@
         <v>8</v>
       </c>
       <c r="C115" t="s">
-        <v>507</v>
+        <v>501</v>
       </c>
       <c r="D115">
         <v>960.73</v>
@@ -10478,7 +10459,7 @@
         <v>22</v>
       </c>
       <c r="C116" t="s">
-        <v>513</v>
+        <v>507</v>
       </c>
       <c r="D116">
         <v>94.38</v>
@@ -10553,7 +10534,7 @@
         <v>22</v>
       </c>
       <c r="C117" t="s">
-        <v>513</v>
+        <v>507</v>
       </c>
       <c r="D117">
         <v>8594.65</v>
@@ -10628,7 +10609,7 @@
         <v>22</v>
       </c>
       <c r="C118" t="s">
-        <v>511</v>
+        <v>505</v>
       </c>
       <c r="D118">
         <v>638.15</v>
@@ -10706,7 +10687,7 @@
         <v>22</v>
       </c>
       <c r="C119" t="s">
-        <v>512</v>
+        <v>506</v>
       </c>
       <c r="D119">
         <v>23.44</v>
@@ -10781,7 +10762,7 @@
         <v>22</v>
       </c>
       <c r="C120" t="s">
-        <v>510</v>
+        <v>504</v>
       </c>
       <c r="D120">
         <v>588.47</v>
@@ -10861,7 +10842,7 @@
         <v>22</v>
       </c>
       <c r="C121" t="s">
-        <v>513</v>
+        <v>507</v>
       </c>
       <c r="D121">
         <v>93.67</v>
@@ -10922,7 +10903,7 @@
         <v>22</v>
       </c>
       <c r="C122" t="s">
-        <v>508</v>
+        <v>502</v>
       </c>
       <c r="D122">
         <v>166.9</v>
@@ -10991,7 +10972,7 @@
         <v>8</v>
       </c>
       <c r="C123" t="s">
-        <v>506</v>
+        <v>500</v>
       </c>
       <c r="D123">
         <v>94.33</v>
@@ -11067,7 +11048,7 @@
         <v>8</v>
       </c>
       <c r="C124" t="s">
-        <v>505</v>
+        <v>499</v>
       </c>
       <c r="D124">
         <v>37.58</v>
@@ -11143,7 +11124,7 @@
         <v>22</v>
       </c>
       <c r="C125" t="s">
-        <v>511</v>
+        <v>505</v>
       </c>
       <c r="D125">
         <v>8420.6</v>
@@ -11216,7 +11197,7 @@
         <v>22</v>
       </c>
       <c r="C126" t="s">
-        <v>509</v>
+        <v>503</v>
       </c>
       <c r="D126">
         <v>498.85</v>
@@ -11292,7 +11273,7 @@
         <v>22</v>
       </c>
       <c r="C127" t="s">
-        <v>508</v>
+        <v>502</v>
       </c>
       <c r="D127">
         <v>11.45</v>
@@ -11363,7 +11344,7 @@
         <v>8</v>
       </c>
       <c r="C128" t="s">
-        <v>507</v>
+        <v>501</v>
       </c>
       <c r="D128">
         <v>4395.9799999999996</v>
@@ -11438,7 +11419,7 @@
         <v>22</v>
       </c>
       <c r="C129" t="s">
-        <v>510</v>
+        <v>504</v>
       </c>
       <c r="D129">
         <v>703.09</v>
@@ -11489,7 +11470,7 @@
         <v>8</v>
       </c>
       <c r="C130" t="s">
-        <v>506</v>
+        <v>500</v>
       </c>
       <c r="D130">
         <v>205.59</v>
@@ -11535,7 +11516,7 @@
         <v>81</v>
       </c>
       <c r="C131" t="s">
-        <v>509</v>
+        <v>503</v>
       </c>
       <c r="D131">
         <v>851.36</v>
@@ -11610,7 +11591,7 @@
         <v>22</v>
       </c>
       <c r="C132" t="s">
-        <v>514</v>
+        <v>508</v>
       </c>
       <c r="D132">
         <v>635.23</v>
@@ -11685,7 +11666,7 @@
         <v>22</v>
       </c>
       <c r="C133" t="s">
-        <v>514</v>
+        <v>508</v>
       </c>
       <c r="D133">
         <v>532.54999999999995</v>
@@ -11760,7 +11741,7 @@
         <v>8</v>
       </c>
       <c r="C134" t="s">
-        <v>507</v>
+        <v>501</v>
       </c>
       <c r="D134">
         <v>390.46</v>
@@ -11834,7 +11815,7 @@
         <v>81</v>
       </c>
       <c r="C135" t="s">
-        <v>512</v>
+        <v>506</v>
       </c>
       <c r="D135">
         <v>342.95</v>
@@ -11907,7 +11888,7 @@
         <v>22</v>
       </c>
       <c r="C136" t="s">
-        <v>512</v>
+        <v>506</v>
       </c>
       <c r="D136">
         <v>90.32</v>
@@ -11982,7 +11963,7 @@
         <v>8</v>
       </c>
       <c r="C137" t="s">
-        <v>506</v>
+        <v>500</v>
       </c>
       <c r="D137">
         <v>91.53</v>
@@ -12055,7 +12036,7 @@
         <v>8</v>
       </c>
       <c r="C138" t="s">
-        <v>507</v>
+        <v>501</v>
       </c>
       <c r="D138">
         <v>37.82</v>
@@ -12131,7 +12112,7 @@
         <v>8</v>
       </c>
       <c r="C139" t="s">
-        <v>505</v>
+        <v>499</v>
       </c>
       <c r="D139">
         <v>99.39</v>
@@ -12175,7 +12156,7 @@
         <v>22</v>
       </c>
       <c r="C140" t="s">
-        <v>511</v>
+        <v>505</v>
       </c>
       <c r="D140">
         <v>635.98</v>
@@ -12216,7 +12197,7 @@
         <v>81</v>
       </c>
       <c r="C141" t="s">
-        <v>509</v>
+        <v>503</v>
       </c>
       <c r="D141">
         <v>51.53</v>
@@ -12294,7 +12275,7 @@
         <v>22</v>
       </c>
       <c r="C142" t="s">
-        <v>510</v>
+        <v>504</v>
       </c>
       <c r="D142">
         <v>63.06</v>
@@ -12369,7 +12350,7 @@
         <v>22</v>
       </c>
       <c r="C143" t="s">
-        <v>512</v>
+        <v>506</v>
       </c>
       <c r="D143">
         <v>6029.5</v>
@@ -12444,7 +12425,7 @@
         <v>22</v>
       </c>
       <c r="C144" t="s">
-        <v>511</v>
+        <v>505</v>
       </c>
       <c r="D144">
         <v>62.75</v>
@@ -12522,7 +12503,7 @@
         <v>22</v>
       </c>
       <c r="C145" t="s">
-        <v>514</v>
+        <v>508</v>
       </c>
       <c r="D145">
         <v>6546.82</v>
@@ -12598,7 +12579,7 @@
         <v>22</v>
       </c>
       <c r="C146" t="s">
-        <v>513</v>
+        <v>507</v>
       </c>
       <c r="D146">
         <v>70.41</v>
@@ -12649,7 +12630,7 @@
         <v>22</v>
       </c>
       <c r="C147" t="s">
-        <v>511</v>
+        <v>505</v>
       </c>
       <c r="D147">
         <v>7110.97</v>
@@ -12722,7 +12703,7 @@
         <v>22</v>
       </c>
       <c r="C148" t="s">
-        <v>509</v>
+        <v>503</v>
       </c>
       <c r="D148">
         <v>804.93</v>
@@ -12798,7 +12779,7 @@
         <v>8</v>
       </c>
       <c r="C149" t="s">
-        <v>505</v>
+        <v>499</v>
       </c>
       <c r="D149">
         <v>3626.28</v>
@@ -12878,7 +12859,7 @@
         <v>22</v>
       </c>
       <c r="C150" t="s">
-        <v>513</v>
+        <v>507</v>
       </c>
       <c r="D150">
         <v>58.77</v>
@@ -12949,7 +12930,7 @@
         <v>81</v>
       </c>
       <c r="C151" t="s">
-        <v>512</v>
+        <v>506</v>
       </c>
       <c r="D151">
         <v>403.67</v>
@@ -13022,7 +13003,7 @@
         <v>22</v>
       </c>
       <c r="C152" t="s">
-        <v>511</v>
+        <v>505</v>
       </c>
       <c r="D152">
         <v>966.76</v>
@@ -13063,7 +13044,7 @@
         <v>8</v>
       </c>
       <c r="C153" t="s">
-        <v>507</v>
+        <v>501</v>
       </c>
       <c r="D153">
         <v>776.39</v>
@@ -13100,7 +13081,7 @@
         <v>22</v>
       </c>
       <c r="C154" t="s">
-        <v>510</v>
+        <v>504</v>
       </c>
       <c r="D154">
         <v>294.23</v>
@@ -13139,7 +13120,7 @@
         <v>22</v>
       </c>
       <c r="C155" t="s">
-        <v>511</v>
+        <v>505</v>
       </c>
       <c r="D155">
         <v>33.409999999999997</v>
@@ -13178,7 +13159,7 @@
         <v>22</v>
       </c>
       <c r="C156" t="s">
-        <v>514</v>
+        <v>508</v>
       </c>
       <c r="D156">
         <v>700.15</v>
@@ -13224,7 +13205,7 @@
         <v>22</v>
       </c>
       <c r="C157" t="s">
-        <v>508</v>
+        <v>502</v>
       </c>
       <c r="D157">
         <v>816.27</v>
@@ -13263,7 +13244,7 @@
         <v>22</v>
       </c>
       <c r="C158" t="s">
-        <v>514</v>
+        <v>508</v>
       </c>
       <c r="D158">
         <v>475.73</v>
@@ -13300,7 +13281,7 @@
         <v>22</v>
       </c>
       <c r="C159" t="s">
-        <v>510</v>
+        <v>504</v>
       </c>
       <c r="D159">
         <v>482.8</v>
@@ -13339,7 +13320,7 @@
         <v>22</v>
       </c>
       <c r="C160" t="s">
-        <v>508</v>
+        <v>502</v>
       </c>
       <c r="D160">
         <v>762.29</v>
@@ -13408,7 +13389,7 @@
         <v>81</v>
       </c>
       <c r="C161" t="s">
-        <v>510</v>
+        <v>504</v>
       </c>
       <c r="D161">
         <v>336.51</v>
@@ -13447,7 +13428,7 @@
         <v>22</v>
       </c>
       <c r="C162" t="s">
-        <v>512</v>
+        <v>506</v>
       </c>
       <c r="D162">
         <v>23.01</v>
@@ -13484,7 +13465,7 @@
         <v>22</v>
       </c>
       <c r="C163" t="s">
-        <v>510</v>
+        <v>504</v>
       </c>
       <c r="D163">
         <v>78.84</v>
@@ -13521,7 +13502,7 @@
         <v>22</v>
       </c>
       <c r="C164" t="s">
-        <v>508</v>
+        <v>502</v>
       </c>
       <c r="D164">
         <v>3353.74</v>
@@ -13562,7 +13543,7 @@
         <v>8</v>
       </c>
       <c r="C165" t="s">
-        <v>505</v>
+        <v>499</v>
       </c>
       <c r="D165">
         <v>71.319999999999993</v>
@@ -13608,7 +13589,7 @@
         <v>8</v>
       </c>
       <c r="C166" t="s">
-        <v>506</v>
+        <v>500</v>
       </c>
       <c r="D166">
         <v>8570.83</v>
@@ -13667,7 +13648,7 @@
         <v>8</v>
       </c>
       <c r="C167" t="s">
-        <v>506</v>
+        <v>500</v>
       </c>
       <c r="D167">
         <v>489.61</v>
@@ -13726,7 +13707,7 @@
         <v>8</v>
       </c>
       <c r="C168" t="s">
-        <v>506</v>
+        <v>500</v>
       </c>
       <c r="D168">
         <v>715.66</v>
@@ -13785,7 +13766,7 @@
         <v>8</v>
       </c>
       <c r="C169" t="s">
-        <v>505</v>
+        <v>499</v>
       </c>
       <c r="D169">
         <v>1902.3</v>
@@ -13831,7 +13812,7 @@
         <v>8</v>
       </c>
       <c r="C170" t="s">
-        <v>506</v>
+        <v>500</v>
       </c>
       <c r="D170">
         <v>9638.59</v>
@@ -13872,7 +13853,7 @@
         <v>22</v>
       </c>
       <c r="C171" t="s">
-        <v>510</v>
+        <v>504</v>
       </c>
       <c r="D171">
         <v>5275.13</v>
@@ -13911,7 +13892,7 @@
         <v>22</v>
       </c>
       <c r="C172" t="s">
-        <v>508</v>
+        <v>502</v>
       </c>
       <c r="D172">
         <v>371.24</v>
@@ -13952,7 +13933,7 @@
         <v>8</v>
       </c>
       <c r="C173" t="s">
-        <v>505</v>
+        <v>499</v>
       </c>
       <c r="D173">
         <v>4947.9399999999996</v>
@@ -13991,7 +13972,7 @@
         <v>8</v>
       </c>
       <c r="C174" t="s">
-        <v>505</v>
+        <v>499</v>
       </c>
       <c r="D174">
         <v>79.150000000000006</v>
@@ -14037,7 +14018,7 @@
         <v>22</v>
       </c>
       <c r="C175" t="s">
-        <v>509</v>
+        <v>503</v>
       </c>
       <c r="D175">
         <v>560.79999999999995</v>
@@ -14096,7 +14077,7 @@
         <v>22</v>
       </c>
       <c r="C176" t="s">
-        <v>512</v>
+        <v>506</v>
       </c>
       <c r="D176">
         <v>586.54</v>
@@ -14147,7 +14128,7 @@
         <v>22</v>
       </c>
       <c r="C177" t="s">
-        <v>514</v>
+        <v>508</v>
       </c>
       <c r="D177">
         <v>3951.16</v>
@@ -14198,7 +14179,7 @@
         <v>81</v>
       </c>
       <c r="C178" t="s">
-        <v>510</v>
+        <v>504</v>
       </c>
       <c r="D178">
         <v>501.99</v>
@@ -14235,7 +14216,7 @@
         <v>8</v>
       </c>
       <c r="C179" t="s">
-        <v>505</v>
+        <v>499</v>
       </c>
       <c r="D179">
         <v>556.99</v>
@@ -14297,7 +14278,7 @@
         <v>8</v>
       </c>
       <c r="C180" t="s">
-        <v>507</v>
+        <v>501</v>
       </c>
       <c r="D180">
         <v>61.92</v>
@@ -14346,7 +14327,7 @@
         <v>81</v>
       </c>
       <c r="C181" t="s">
-        <v>508</v>
+        <v>502</v>
       </c>
       <c r="D181">
         <v>152.86000000000001</v>
@@ -14405,7 +14386,7 @@
         <v>22</v>
       </c>
       <c r="C182" t="s">
-        <v>514</v>
+        <v>508</v>
       </c>
       <c r="D182">
         <v>59.78</v>
@@ -14442,7 +14423,7 @@
         <v>22</v>
       </c>
       <c r="C183" t="s">
-        <v>514</v>
+        <v>508</v>
       </c>
       <c r="D183">
         <v>157.5</v>
@@ -14479,7 +14460,7 @@
         <v>22</v>
       </c>
       <c r="C184" t="s">
-        <v>514</v>
+        <v>508</v>
       </c>
       <c r="D184">
         <v>46.2</v>
@@ -14525,7 +14506,7 @@
         <v>22</v>
       </c>
       <c r="C185" t="s">
-        <v>509</v>
+        <v>503</v>
       </c>
       <c r="D185">
         <v>4935.3900000000003</v>
@@ -14562,7 +14543,7 @@
         <v>8</v>
       </c>
       <c r="C186" t="s">
-        <v>506</v>
+        <v>500</v>
       </c>
       <c r="D186">
         <v>80.930000000000007</v>
@@ -14601,7 +14582,7 @@
         <v>8</v>
       </c>
       <c r="C187" t="s">
-        <v>506</v>
+        <v>500</v>
       </c>
       <c r="D187">
         <v>626.75</v>
@@ -14638,7 +14619,7 @@
         <v>22</v>
       </c>
       <c r="C188" t="s">
-        <v>514</v>
+        <v>508</v>
       </c>
       <c r="D188">
         <v>639.17999999999995</v>
@@ -14679,7 +14660,7 @@
         <v>22</v>
       </c>
       <c r="C189" t="s">
-        <v>509</v>
+        <v>503</v>
       </c>
       <c r="D189">
         <v>6678.39</v>
@@ -14716,7 +14697,7 @@
         <v>22</v>
       </c>
       <c r="C190" t="s">
-        <v>509</v>
+        <v>503</v>
       </c>
       <c r="D190">
         <v>17.8</v>
@@ -14753,7 +14734,7 @@
         <v>81</v>
       </c>
       <c r="C191" t="s">
-        <v>512</v>
+        <v>506</v>
       </c>
       <c r="D191">
         <v>685.78</v>
@@ -14799,7 +14780,7 @@
         <v>22</v>
       </c>
       <c r="C192" t="s">
-        <v>511</v>
+        <v>505</v>
       </c>
       <c r="D192">
         <v>6117.91</v>
@@ -14836,7 +14817,7 @@
         <v>22</v>
       </c>
       <c r="C193" t="s">
-        <v>509</v>
+        <v>503</v>
       </c>
       <c r="D193">
         <v>178.33</v>
@@ -14873,7 +14854,7 @@
         <v>8</v>
       </c>
       <c r="C194" t="s">
-        <v>505</v>
+        <v>499</v>
       </c>
       <c r="D194">
         <v>7409.26</v>
@@ -14910,7 +14891,7 @@
         <v>8</v>
       </c>
       <c r="C195" t="s">
-        <v>506</v>
+        <v>500</v>
       </c>
       <c r="D195">
         <v>417.42</v>
@@ -14969,7 +14950,7 @@
         <v>22</v>
       </c>
       <c r="C196" t="s">
-        <v>514</v>
+        <v>508</v>
       </c>
       <c r="D196">
         <v>669.3</v>
@@ -15010,7 +14991,7 @@
         <v>81</v>
       </c>
       <c r="C197" t="s">
-        <v>509</v>
+        <v>503</v>
       </c>
       <c r="D197">
         <v>9641.58</v>
@@ -15047,7 +15028,7 @@
         <v>22</v>
       </c>
       <c r="C198" t="s">
-        <v>514</v>
+        <v>508</v>
       </c>
       <c r="D198">
         <v>63.6</v>
@@ -15088,7 +15069,7 @@
         <v>8</v>
       </c>
       <c r="C199" t="s">
-        <v>506</v>
+        <v>500</v>
       </c>
       <c r="D199">
         <v>430.86</v>
@@ -15125,7 +15106,7 @@
         <v>81</v>
       </c>
       <c r="C200" t="s">
-        <v>508</v>
+        <v>502</v>
       </c>
       <c r="D200">
         <v>194.72</v>
@@ -15176,7 +15157,7 @@
         <v>8</v>
       </c>
       <c r="C201" t="s">
-        <v>505</v>
+        <v>499</v>
       </c>
       <c r="D201">
         <v>4419.24</v>
@@ -15237,63 +15218,6 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K1"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
-  <cols>
-    <col min="1" max="1" width="7.796875" customWidth="1"/>
-    <col min="2" max="2" width="7.296875" customWidth="1"/>
-    <col min="3" max="3" width="7.69921875" customWidth="1"/>
-    <col min="4" max="5" width="11" customWidth="1"/>
-    <col min="6" max="6" width="10.8984375" customWidth="1"/>
-    <col min="7" max="7" width="9.3984375" customWidth="1"/>
-    <col min="8" max="8" width="8.8984375" customWidth="1"/>
-    <col min="9" max="9" width="11" customWidth="1"/>
-    <col min="10" max="10" width="8.5" customWidth="1"/>
-    <col min="11" max="11" width="7" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:11" ht="27.6">
-      <c r="A1" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>488</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>489</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>490</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>491</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>492</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>493</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>79</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B11"/>
   <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
@@ -15303,15 +15227,15 @@
   <sheetData>
     <row r="1" spans="1:2" ht="27.6">
       <c r="A1" s="1" t="s">
-        <v>494</v>
+        <v>488</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>495</v>
+        <v>489</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>496</v>
+        <v>490</v>
       </c>
       <c r="B2">
         <v>200</v>
@@ -15319,7 +15243,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>497</v>
+        <v>491</v>
       </c>
       <c r="B3">
         <v>65</v>
@@ -15327,7 +15251,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>498</v>
+        <v>492</v>
       </c>
       <c r="B4">
         <v>35</v>
@@ -15343,7 +15267,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>499</v>
+        <v>493</v>
       </c>
       <c r="B6">
         <v>90</v>
@@ -15351,7 +15275,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>500</v>
+        <v>494</v>
       </c>
       <c r="B7">
         <v>60</v>
@@ -15359,7 +15283,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
-        <v>501</v>
+        <v>495</v>
       </c>
       <c r="B8">
         <v>120</v>
@@ -15367,7 +15291,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" t="s">
-        <v>502</v>
+        <v>496</v>
       </c>
       <c r="B9">
         <v>20</v>
@@ -15375,7 +15299,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" t="s">
-        <v>503</v>
+        <v>497</v>
       </c>
       <c r="B10">
         <v>20</v>
@@ -15383,7 +15307,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" t="s">
-        <v>504</v>
+        <v>498</v>
       </c>
       <c r="B11">
         <v>35</v>

</xml_diff>